<commit_message>
Usa gramas e unidades da tabela do PDF nos itens novos
Granulado 400 g, chocolate 50% 200 g, pote 150 ml 25 un e
barra de chocolate 1000 g — mesmos conteúdos da compra inicial.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/planilha_custos_confeitaria_atualizada.xlsx
+++ b/planilha_custos_confeitaria_atualizada.xlsx
@@ -1942,11 +1942,11 @@
         <v>19.99</v>
       </c>
       <c r="D40" s="44" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="E40" s="42" t="inlineStr">
         <is>
-          <t>pacote</t>
+          <t>gramas</t>
         </is>
       </c>
       <c r="F40" s="45">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G40" s="42" t="inlineStr">
         <is>
-          <t>Quarta compra (peso do pacote não informado)</t>
+          <t>Quarta compra</t>
         </is>
       </c>
     </row>
@@ -1974,11 +1974,11 @@
         <v>38.99</v>
       </c>
       <c r="D41" s="44" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="E41" s="42" t="inlineStr">
         <is>
-          <t>pacote</t>
+          <t>gramas</t>
         </is>
       </c>
       <c r="F41" s="45">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="G41" s="42" t="inlineStr">
         <is>
-          <t>Quarta compra (peso do pacote não informado)</t>
+          <t>Quarta compra</t>
         </is>
       </c>
     </row>
@@ -2198,11 +2198,11 @@
         <v>11.59</v>
       </c>
       <c r="D48" s="39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E48" s="37" t="inlineStr">
         <is>
-          <t>pacote</t>
+          <t>unidades</t>
         </is>
       </c>
       <c r="F48" s="40">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="G48" s="37" t="inlineStr">
         <is>
-          <t>Quinta compra (qtd. do pacote não informada)</t>
+          <t>Quinta compra</t>
         </is>
       </c>
     </row>
@@ -2390,11 +2390,11 @@
         <v>30</v>
       </c>
       <c r="D54" s="44" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E54" s="42" t="inlineStr">
         <is>
-          <t>unidade</t>
+          <t>gramas</t>
         </is>
       </c>
       <c r="F54" s="45">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="G54" s="42" t="inlineStr">
         <is>
-          <t>Sexta compra (peso não informado)</t>
+          <t>Sexta compra</t>
         </is>
       </c>
     </row>

</xml_diff>